<commit_message>
feat: Add Holiday & Leaves Calendar system with date-grouped Excel exports
- Added data/holidays.json database for custom leaves/festivals/events
- New REST API endpoints: GET/POST /api/holidays, DELETE /api/holidays/:id
- Secured /api/holidays under X-Auth-Token middleware
- Refactored saveDiskExcel() into generateStyledWorkbook(reports, holidays)
  - Groups rows by date (newest first)
  - Auto-detects Sundays (Weekly Off) and India national holidays
  - Inserts amber-highlighted holiday/leave banner rows per date
  - Adds 2 blank spacer rows between each date group
- Updated POST /api/reports/export to use same grouped workbook logic
- Added 'Holidays & Leaves' tab panel in dashboard.html
  - Form to declare Personal Leave, Festival Holiday, Company Event
  - Live table showing all declared holidays with delete action
- dashboard.js: Tab switching, fetchHolidays(), renderHolidaysTable(), deleteHoliday(), form submit logic
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="All Call Reports" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Call Reports Log" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -697,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -968,73 +968,23 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>13</v>
@@ -1043,24 +993,24 @@
         <v>61</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>73</v>
+        <v>39</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>13</v>
@@ -1069,6 +1019,58 @@
         <v>61</v>
       </c>
       <c r="H14" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Wrap mobile holiday listeners in null guards to prevent app.js crash
- Root cause: holiday element listeners were calling .addEventListener() directly
  without null checks, causing 'Cannot read properties of null' TypeError
- This crashed the entire DOMContentLoaded handler, which stopped form submission,
  department loading, and all other mobile features from working
- Fix: Wrap all 4 holiday event listeners (mobileAddHolidayBtn, cancelMobileHolidayBtn,
  mobileHolidayType, saveMobileHolidayBtn) in if(element) null guards
- All inner element accesses also guarded with conditional checks
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="83">
   <si>
     <t>Date</t>
   </si>
@@ -37,6 +37,30 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>2026-07-06T16:42</t>
+  </si>
+  <si>
+    <t>Bhavin soni</t>
+  </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>CMOS cell error date and time mismatch</t>
+  </si>
+  <si>
+    <t>Change CMOS cell and date and time set</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>2026-07-06T15:31</t>
   </si>
   <si>
@@ -52,24 +76,12 @@
     <t>Server login and sql database open</t>
   </si>
   <si>
-    <t>Resolved</t>
-  </si>
-  <si>
-    <t>2026-07-06</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>2026-07-06T14:27</t>
   </si>
   <si>
     <t>Sejal parik</t>
   </si>
   <si>
-    <t>Service</t>
-  </si>
-  <si>
     <t>Video link</t>
   </si>
   <si>
@@ -160,10 +172,16 @@
     <t>Simit</t>
   </si>
   <si>
+    <t>Spear P5</t>
+  </si>
+  <si>
     <t>PC  not working no startup</t>
   </si>
   <si>
     <t>I will check pc plugin chack other switches but till not working</t>
+  </si>
+  <si>
+    <t>2026-07-07</t>
   </si>
   <si>
     <t>Give other pc  13 buyback system</t>
@@ -697,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -794,13 +812,13 @@
         <v>22</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>13</v>
@@ -814,19 +832,19 @@
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>13</v>
@@ -835,24 +853,24 @@
         <v>14</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>13</v>
@@ -861,24 +879,24 @@
         <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>13</v>
@@ -887,18 +905,18 @@
         <v>14</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>44</v>
@@ -913,24 +931,24 @@
         <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>13</v>
@@ -939,18 +957,18 @@
         <v>14</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>54</v>
@@ -962,40 +980,40 @@
         <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="H11" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
+    <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>63</v>
@@ -1004,7 +1022,7 @@
         <v>64</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>65</v>
@@ -1016,33 +1034,33 @@
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>15</v>
@@ -1050,28 +1068,54 @@
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>76</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Complete rebuild of index.html and app.js
- index.html: Fixed missing form tag (was root cause of form not submitting)
  All form fields (Date, User, Department, Problems, Action, Status, Remarks)
  are now properly inside <form id='callForm'>
  Proper semantic structure with <main> containing the form
  All element IDs verified and matched to app.js references

- app.js: Full clean rewrite - every DOM binding null-guarded
  Auth flow: initAuth -> unlockApp() on success
  Form submit: complete online/offline handling
  Departments: fetch + populate + add new department
  Active reports: fetch, render, edit mode
  Voice dictation: null-safe setup
  Theme toggle, inactivity timer, offline queue all working
  Forgot PIN modal, Change PIN modal fully functional
  Holidays & Leaves: fetch, render, add, delete - all null-guarded

- PIN reset to VashLogger@2026! (server will auto-hash on startup)
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="88">
   <si>
     <t>Date</t>
   </si>
@@ -37,6 +37,27 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>2026-07-07T10:51</t>
+  </si>
+  <si>
+    <t>Kunal ghotikar</t>
+  </si>
+  <si>
+    <t>Spear P5</t>
+  </si>
+  <si>
+    <t>HHD not detected and pc not responding show</t>
+  </si>
+  <si>
+    <t>HHD change and other give but still same problem  HHD It table</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>2026-07-06T16:42</t>
   </si>
   <si>
@@ -58,9 +79,6 @@
     <t>2026-07-06</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>2026-07-06T15:31</t>
   </si>
   <si>
@@ -170,9 +188,6 @@
   </si>
   <si>
     <t>Simit</t>
-  </si>
-  <si>
-    <t>Spear P5</t>
   </si>
   <si>
     <t>PC  not working no startup</t>
@@ -266,7 +281,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -286,12 +301,18 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF92400E"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF065F46"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,6 +327,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -356,7 +382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -375,6 +401,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -715,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -775,245 +804,245 @@
         <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    </row>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>13</v>
+        <v>19</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>13</v>
+        <v>26</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>13</v>
+        <v>30</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>13</v>
+        <v>35</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>13</v>
+        <v>40</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>13</v>
+        <v>45</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="H11" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>63</v>
@@ -1022,7 +1051,7 @@
         <v>64</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>65</v>
@@ -1030,92 +1059,120 @@
       <c r="E14" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>13</v>
+      <c r="F14" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="G14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    </row>
+    <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="F18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="B19" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="C19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H17" s="6" t="s">
+      <c r="F19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>82</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Expose Mobile App and Dashboard App on separate ports with configurable local network IP
- Separated ports: Port 3000 serves NIK Call Report (Mobile App), Port 3001 serves IT-Daily Call Report Dashboard (PC Admin).
- Forbidden dashboard access on Mobile port 3000 to improve local network separation.
- Added data/network_config.json supporting custom binding IP, mobilePort, dashboardPort, allowed Windows users, and AD Auth toggle.
- Implemented lightweight Windows authentication/domain groups check using CLI (whoami) for Port 3001.
- Setup dual Express listeners: appMobile and appDashboard binding safely to network interfaces.
- Updated all existing API logic to function correctly with dual port database sharing.
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="92">
   <si>
     <t>Date</t>
   </si>
@@ -37,6 +37,30 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>2026-07-07T10:57</t>
+  </si>
+  <si>
+    <t>Vijay b</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Solid edge problem assembly link damage</t>
+  </si>
+  <si>
+    <t>So call Aarti bhaskar and problem solved but tc talk to problem is system high priority set  but assembly load more time</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>2026-07-07</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>2026-07-07T10:51</t>
   </si>
   <si>
@@ -55,9 +79,6 @@
     <t>In Progress</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>2026-07-06T16:42</t>
   </si>
   <si>
@@ -73,9 +94,6 @@
     <t>Change CMOS cell and date and time set</t>
   </si>
   <si>
-    <t>Resolved</t>
-  </si>
-  <si>
     <t>2026-07-06</t>
   </si>
   <si>
@@ -160,9 +178,6 @@
     <t>Rashmikant joshi</t>
   </si>
   <si>
-    <t>Design</t>
-  </si>
-  <si>
     <t>Outlook problem</t>
   </si>
   <si>
@@ -194,9 +209,6 @@
   </si>
   <si>
     <t>I will check pc plugin chack other switches but till not working</t>
-  </si>
-  <si>
-    <t>2026-07-07</t>
   </si>
   <si>
     <t>Give other pc  13 buyback system</t>
@@ -301,13 +313,13 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF92400E"/>
+      <color rgb="FF065F46"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF065F46"/>
+      <color rgb="FF92400E"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
@@ -331,12 +343,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFD1FAE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD1FAE5"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -744,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -804,37 +816,37 @@
         <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
+    <row r="5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
@@ -851,92 +863,92 @@
       <c r="E6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>20</v>
+      <c r="F6" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>21</v>
-      </c>
       <c r="H7" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>20</v>
+        <v>36</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>20</v>
+        <v>41</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -947,33 +959,33 @@
         <v>43</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>20</v>
+        <v>46</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>50</v>
@@ -981,40 +993,40 @@
       <c r="E11" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>20</v>
+      <c r="F11" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>20</v>
+        <v>56</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1025,7 +1037,7 @@
         <v>58</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>59</v>
@@ -1033,94 +1045,94 @@
       <c r="E13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>20</v>
+      <c r="F13" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="3" t="s">
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
     <row r="16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
+    <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1131,7 +1143,7 @@
         <v>79</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>80</v>
@@ -1139,14 +1151,14 @@
       <c r="E19" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>20</v>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1157,22 +1169,48 @@
         <v>83</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H20" s="3" t="s">
+      <c r="B21" s="6" t="s">
         <v>87</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Integrate Windows User Session and Active Directory domain validation for Dashboard (Port 3001)
- Enhanced windowsAuthMiddleware to check both whoami username and whoami /groups.
- Configured network_config.json to enable AD/Windows authentication.
- Restricts port 3001 access to specified domain groups, domain administrators, or specified standard users.
- Accessing from unauthorized user returns a detailed 403 Forbidden with credential identity feedback.
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -40,13 +40,13 @@
     <t>2026-07-07T10:57</t>
   </si>
   <si>
-    <t>Vijay b</t>
+    <t>Vijay bhatt</t>
   </si>
   <si>
     <t>Design</t>
   </si>
   <si>
-    <t>Solid edge problem assembly link damage</t>
+    <t>Assembly link borken in solid edge</t>
   </si>
   <si>
     <t>So call Aarti bhaskar and problem solved but tc talk to problem is system high priority set  but assembly load more time</t>
@@ -115,13 +115,13 @@
     <t>2026-07-06T14:27</t>
   </si>
   <si>
-    <t>Sejal parik</t>
+    <t>Sejal parikh</t>
   </si>
   <si>
     <t>Video link</t>
   </si>
   <si>
-    <t>Create video link and send saje ma&amp;#x27;am and manoj Agarwal</t>
+    <t>Create video link and send saje ma&amp;amp;#x27;am and manoj Agarwal</t>
   </si>
   <si>
     <t>2026-07-06T13:49</t>
@@ -202,7 +202,7 @@
     <t>2026-07-06T11:14</t>
   </si>
   <si>
-    <t>Simit</t>
+    <t>Smit Patel</t>
   </si>
   <si>
     <t>PC  not working no startup</t>
@@ -217,7 +217,7 @@
     <t>2026-07-06T11:07</t>
   </si>
   <si>
-    <t>Kunal ghoyikat</t>
+    <t>Kunal Ghotikar</t>
   </si>
   <si>
     <t>Outlook and folder shortcuts create</t>
@@ -1063,7 +1063,7 @@
         <v>63</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
🚀 Complete Overhaul: AI Grammar Polish, Firebase Auth & Smooth UI Animations
This mega-commit introduces several advanced features to the Call Logger application:

✨ AI Grammar & Translation Engine: Integrated Google Gemini AI to instantly translate Hindi voice dictation to flawless English, and gracefully auto-correct any typed text.

🔐 Robust Firebase Authentication: Successfully migrated the entire platform away from the legacy local Windows Domain/PIN system. Now features fully secure email/password auth using Firebase.

🔄 Intelligent Dual-Port Redirection: Fixed complex cross-origin 'Forbidden' port errors by implementing graceful server-side redirects on Port 3000.

🎨 Premium Glassmorphic UI: Completely revamped the user interface with dark mode aesthetics, smooth micro-animations, animated waveform bars for voice recording, and stunning gradient effects.

🐛 General Polish: Cleaned up deprecated server dependencies and enhanced rate limiting.
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="110">
   <si>
     <t>Date</t>
   </si>
@@ -37,28 +37,43 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>2026-07-08T11:42</t>
+  </si>
+  <si>
+    <t>Parth</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Disk storage full</t>
+  </si>
+  <si>
+    <t>Clean disk storage and fix all problems</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>2026-07-07T14:38</t>
   </si>
   <si>
     <t>Chaitnya</t>
   </si>
   <si>
-    <t>Design</t>
-  </si>
-  <si>
     <t>Required bullzip</t>
   </si>
   <si>
     <t>Install new bullzip software...</t>
   </si>
   <si>
-    <t>Resolved</t>
-  </si>
-  <si>
     <t>2026-07-07</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>2026-07-07T14:37</t>
@@ -795,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -858,79 +873,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>15</v>
@@ -938,32 +903,82 @@
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>34</v>
+        <v>25</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>35</v>
@@ -972,97 +987,47 @@
         <v>36</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="G9" s="5" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    <row r="10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>15</v>
@@ -1070,77 +1035,77 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>65</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>15</v>
@@ -1148,84 +1113,134 @@
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="3" t="s">
+      <c r="F20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>85</v>
@@ -1234,7 +1249,7 @@
         <v>86</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>87</v>
@@ -1246,88 +1261,116 @@
         <v>13</v>
       </c>
       <c r="G21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    </row>
+    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="F25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="C26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H24" s="3" t="s">
+      <c r="F26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>104</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add comprehensive Bills management and Excel export sync
- Added full Bills management module to dashboard with all 11 columns (Bill Date, Ref.Code, Challan No, Supplier, Item Desc, Qty, Amount, PO Number, Purpose, Remarks, Hand Over).
- Upgraded 'Item Description' field to a multiline textarea to allow freeform typing (Ctrl+Enter support).
- Adjusted CSS grid and table styles to support text wrapping (pre-wrap) for lengthy columns.
- Implemented automated backup script (generate_backups.js) to sync JSON data to CSV and Excel formats.
- Created data migration scripts (migrate_bills_all.js) to import legacy Excel data and support rich text decoding.
- Integrated Ref.Code field successfully across frontend form, table UI, and backend POST API.
</commit_message>
<xml_diff>
--- a/data/reports.xlsx
+++ b/data/reports.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="154">
   <si>
     <t>Date</t>
   </si>
@@ -37,30 +37,147 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>2026-07-09T16:25</t>
+  </si>
+  <si>
+    <t>NIKHIL IT</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Resolving the HDD issues for Kalpesh Trivedi and Kunal Ghotikar.</t>
+  </si>
+  <si>
+    <t>Today, I was troubleshooting an HDD problem. The hard drive was neither showing up nor being detected. Despite applying standard troubleshooting steps, the problem remained unresolved, and the HDD was subsequently scrapped.</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-07-09T16:23</t>
+  </si>
+  <si>
+    <t>Vipul patel</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>A new mouse pad is required.</t>
+  </si>
+  <si>
+    <t>I was given a new mouse pad.</t>
+  </si>
+  <si>
+    <t>2026-07-09T16:20</t>
+  </si>
+  <si>
+    <t>Prakash patel</t>
+  </si>
+  <si>
+    <t>Teamcenter is not opening.</t>
+  </si>
+  <si>
+    <t>I checked and confirmed that Teamcenter had been deleted. I attempted to reinstall it but encountered a problem. After speaking with Dharmesh, the issue was resolved, and Teamcenter is now running properly.</t>
+  </si>
+  <si>
+    <t>2026-07-09T16:18</t>
+  </si>
+  <si>
+    <t>Vishal shilewant</t>
+  </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>The Word file is not printing, and the printer is unresponsive.</t>
+  </si>
+  <si>
+    <t>I will reinstall Microsoft Office and then print properly.</t>
+  </si>
+  <si>
+    <t>2026-07-09T16:15</t>
+  </si>
+  <si>
+    <t>Parth</t>
+  </si>
+  <si>
+    <t>Festo software is required.</t>
+  </si>
+  <si>
+    <t>The new Festo software has been installed and is functioning correctly.</t>
+  </si>
+  <si>
+    <t>2026-07-09T16:09</t>
+  </si>
+  <si>
+    <t>Mukund maida</t>
+  </si>
+  <si>
+    <t>Solid Edge is not working.</t>
+  </si>
+  <si>
+    <t>Please contact TeamCenter Support to resolve the issue.</t>
+  </si>
+  <si>
+    <t>2026-07-09T09:57</t>
+  </si>
+  <si>
+    <t>Chinmay alekar</t>
+  </si>
+  <si>
+    <t>The drawing will not open in AutoCAD. I have tested it on another PC, and the same problem persists.</t>
+  </si>
+  <si>
+    <t>I checked AutoCAD and performed a repair. When I subsequently attempted to open the drawing, it failed. Therefore, I uninstalled and reinstalled AutoCAD 2008.</t>
+  </si>
+  <si>
+    <t>2026-07-08T16:43</t>
+  </si>
+  <si>
+    <t>Kishan</t>
+  </si>
+  <si>
+    <t>There is a problem checking in a part in Teamcenter.</t>
+  </si>
+  <si>
+    <t>I contacted Teamcenter support and spoke with Aarti Bhaskar. She troubleshooted and successfully resolved the issue.</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>2026-07-08T14:20</t>
+  </si>
+  <si>
+    <t>Parag patel</t>
+  </si>
+  <si>
+    <t>P3 Qc</t>
+  </si>
+  <si>
+    <t>I am experiencing an issue with my mouse.</t>
+  </si>
+  <si>
+    <t>I have provided a new mouse and a mouse pad.</t>
+  </si>
+  <si>
     <t>2026-07-08T11:42</t>
   </si>
   <si>
-    <t>Parth</t>
-  </si>
-  <si>
-    <t>Design</t>
-  </si>
-  <si>
     <t>Disk storage full</t>
   </si>
   <si>
     <t>Clean disk storage and fix all problems</t>
   </si>
   <si>
-    <t>Resolved</t>
-  </si>
-  <si>
-    <t>2026-07-08</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>2026-07-07T14:38</t>
   </si>
   <si>
@@ -124,10 +241,13 @@
     <t>Kunal ghotikar</t>
   </si>
   <si>
-    <t>HDD not detected and pc not responding show</t>
-  </si>
-  <si>
-    <t>HDD change and other give but still same problem  HHD It table</t>
+    <t>Spear P5</t>
+  </si>
+  <si>
+    <t>The hard drive is not detected, and the PC is unresponsive.</t>
+  </si>
+  <si>
+    <t>The hard drive was replaced, and other troubleshooting steps were attempted, but the problem persists. The issue might be with the HDD&amp;amp;#x27;s SATA cable.</t>
   </si>
   <si>
     <t>In Progress</t>
@@ -139,9 +259,6 @@
     <t>Bhavin soni</t>
   </si>
   <si>
-    <t>Service</t>
-  </si>
-  <si>
     <t>CMOS cell error date and time mismatch</t>
   </si>
   <si>
@@ -341,13 +458,28 @@
   </si>
   <si>
     <t>Under observation</t>
+  </si>
+  <si>
+    <t>2026-07-02T11:14</t>
+  </si>
+  <si>
+    <t>Kalpesh trivedi</t>
+  </si>
+  <si>
+    <t>The HDD is not detected.</t>
+  </si>
+  <si>
+    <t>Perform all troubleshooting steps. If the hard drive is not detected, retrieve a replacement hard drive from the IT table.</t>
+  </si>
+  <si>
+    <t>Pending</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -377,8 +509,14 @@
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF991B1B"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -403,6 +541,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -448,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -469,6 +612,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -810,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -873,29 +1019,79 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="5" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>15</v>
@@ -903,25 +1099,25 @@
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>15</v>
@@ -929,105 +1125,105 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="6" t="s">
+    <row r="9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>15</v>
@@ -1035,287 +1231,237 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="H13" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
+    <row r="14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>65</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B23" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="3" t="s">
+      <c r="C23" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E23" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H20" s="3" t="s">
+      <c r="F23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="21" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="H23" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
     <row r="24" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>95</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>15</v>
@@ -1323,25 +1469,25 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>15</v>
@@ -1349,28 +1495,292 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="6" t="s">
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="B28" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="C28" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E28" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="H27" s="6" t="s">
+      <c r="F28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="3" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>